<commit_message>
Update Commander HUD, presentation performance and network documentation
Implement living-soldier HUD summaries, optimized unit rings, input validation, performance tooling, and project documentation.

Include current gameplay, navigation, tuning and data updates. Extend local artifact ignores and stop tracking ZCode session files. Keep the oversized prototype map and marketplace-derived Crowd assets local.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>id</t>
   </si>
@@ -68,6 +68,9 @@
   </si>
   <si>
     <t>/Game/Commander/Units/SM_CommanderFourFRobot.SM_CommanderFourFRobot</t>
+  </si>
+  <si>
+    <t>/Game/Commander/Units/SM_CommanderFourFRobot_Crowd.SM_CommanderFourFRobot_Crowd</t>
   </si>
 </sst>
 </file>
@@ -510,7 +513,7 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G4">
         <v>0</v>

</xml_diff>

<commit_message>
Implement commander combat, navigation, and selection systems
Add the army skill bridge, sweep combat, float health, protocol v6 move planning, commander camera and navigation stabilization, selection UI, diagnostics, tests, data assets, and documentation. Disable client positional move prediction that caused visible pullback.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -4,17 +4,19 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Soldiers" sheetId="2" r:id="rId4"/>
+    <sheet name="Skills" sheetId="3" r:id="rId6"/>
+    <sheet name="UnitSkills" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
   <si>
     <t>id</t>
   </si>
@@ -71,6 +73,102 @@
   </si>
   <si>
     <t>/Game/Commander/Units/SM_CommanderFourFRobot_Crowd.SM_CommanderFourFRobot_Crowd</t>
+  </si>
+  <si>
+    <t>扫射调试兵种A；数值非平衡定案</t>
+  </si>
+  <si>
+    <t>TestSoldierB</t>
+  </si>
+  <si>
+    <t>扫射调试兵种B；浮点生命和多兵种验证</t>
+  </si>
+  <si>
+    <t>SkillId</t>
+  </si>
+  <si>
+    <t>DisplayName</t>
+  </si>
+  <si>
+    <t>ExecutorId</t>
+  </si>
+  <si>
+    <t>Tags</t>
+  </si>
+  <si>
+    <t>Strafe</t>
+  </si>
+  <si>
+    <t>单体直接伤害；不接视觉表现</t>
+  </si>
+  <si>
+    <t>扫射</t>
+  </si>
+  <si>
+    <t>DirectSingleTarget</t>
+  </si>
+  <si>
+    <t>Skill.Attack.Basic;Skill.Usage.Common;Weapon.MachineGun</t>
+  </si>
+  <si>
+    <t>StrafeTest</t>
+  </si>
+  <si>
+    <t>替换接口测试；不是正式火炮</t>
+  </si>
+  <si>
+    <t>扫射测试变体</t>
+  </si>
+  <si>
+    <t>Skill.Attack.Basic;Skill.Usage.Common;Weapon.Test</t>
+  </si>
+  <si>
+    <t>UnitTypeId</t>
+  </si>
+  <si>
+    <t>SlotId</t>
+  </si>
+  <si>
+    <t>bDefault</t>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>AttackRatePerSecond</t>
+  </si>
+  <si>
+    <t>RangeCentimeters</t>
+  </si>
+  <si>
+    <t>bool</t>
+  </si>
+  <si>
+    <t>SoldierA_Strafe</t>
+  </si>
+  <si>
+    <t>A默认普攻</t>
+  </si>
+  <si>
+    <t>BasicAttack</t>
+  </si>
+  <si>
+    <t>SoldierB_Strafe</t>
+  </si>
+  <si>
+    <t>B默认普攻</t>
+  </si>
+  <si>
+    <t>SoldierA_Test</t>
+  </si>
+  <si>
+    <t>A替换验证</t>
+  </si>
+  <si>
+    <t>SoldierB_Test</t>
+  </si>
+  <si>
+    <t>B替换验证</t>
   </si>
 </sst>
 </file>
@@ -406,7 +504,7 @@
     <col customWidth="true" max="1" min="1" width="10"/>
     <col customWidth="true" max="2" min="2" width="22"/>
     <col customWidth="true" max="3" min="3" width="46"/>
-    <col customWidth="true" max="9" min="4" width="28"/>
+    <col customWidth="true" max="7" min="4" width="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -429,13 +527,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2">
@@ -452,7 +544,7 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
         <v>12</v>
@@ -460,12 +552,270 @@
       <c r="G2" t="s">
         <v>11</v>
       </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4">
+        <v>3600</v>
+      </c>
+      <c r="E4">
+        <v>100</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5">
+        <v>3600</v>
+      </c>
+      <c r="E5">
+        <v>300.5</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>41</v>
+      </c>
       <c r="H2" t="s">
         <v>11</v>
       </c>
       <c r="I2" t="s">
         <v>11</v>
       </c>
+      <c r="J2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -495,34 +845,136 @@
       <c r="I3" t="s">
         <v>13</v>
       </c>
+      <c r="J3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+      <c r="I4">
+        <v>2</v>
+      </c>
+      <c r="J4">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G5" t="b">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>7.5</v>
+      </c>
+      <c r="I5">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" t="b">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>25</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" t="s">
+        <v>31</v>
+      </c>
+      <c r="G7" t="b">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>15</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4">
-        <v>3600</v>
-      </c>
-      <c r="E4">
-        <v>100</v>
-      </c>
-      <c r="F4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>0</v>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>18000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: advance ship combat and project tooling
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -4,19 +4,21 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Soldiers" sheetId="2" r:id="rId4"/>
     <sheet name="Skills" sheetId="3" r:id="rId6"/>
     <sheet name="UnitSkills" sheetId="4" r:id="rId7"/>
+    <sheet name="SpellFields" sheetId="5" r:id="rId8"/>
+    <sheet name="WeaponMounts" sheetId="6" r:id="rId9"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="104">
   <si>
     <t>id</t>
   </si>
@@ -169,6 +171,165 @@
   </si>
   <si>
     <t>B替换验证</t>
+  </si>
+  <si>
+    <t>WM01</t>
+  </si>
+  <si>
+    <t>WM01 第二兵种；首版沿用调试数值，尚未平衡</t>
+  </si>
+  <si>
+    <t>/Game/Commander/Units/SM_WM01_Crowd.SM_WM01_Crowd</t>
+  </si>
+  <si>
+    <t>WM01_Strafe</t>
+  </si>
+  <si>
+    <t>WM01 默认普攻</t>
+  </si>
+  <si>
+    <t>WM01_Test</t>
+  </si>
+  <si>
+    <t>WM01 替换验证</t>
+  </si>
+  <si>
+    <t>机枪即时单体伤害与枪火表现</t>
+  </si>
+  <si>
+    <t>WM01_HomingMissile</t>
+  </si>
+  <si>
+    <t>独立自动导弹；爆炸由独立法术场结算；调试初值</t>
+  </si>
+  <si>
+    <t>WM01导弹</t>
+  </si>
+  <si>
+    <t>LaunchProjectile</t>
+  </si>
+  <si>
+    <t>Skill.Attack.Basic;Skill.Usage.Common;Weapon.Missile</t>
+  </si>
+  <si>
+    <t>WM01_MissileLauncher</t>
+  </si>
+  <si>
+    <t>默认解锁；3秒/枚，30伤害，150米射程；调试初值非最终平衡</t>
+  </si>
+  <si>
+    <t>MissileLauncher</t>
+  </si>
+  <si>
+    <t>EffectConfigId</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>WM01_MissileExplosion</t>
+  </si>
+  <si>
+    <t>默认解锁；3秒/枚，伤害由SpellFields表提供，150米射程；调试初值非最终平衡</t>
+  </si>
+  <si>
+    <t>RadiusCentimeters</t>
+  </si>
+  <si>
+    <t>Timing</t>
+  </si>
+  <si>
+    <t>DelaySeconds</t>
+  </si>
+  <si>
+    <t>DurationSeconds</t>
+  </si>
+  <si>
+    <t>PulseIntervalSeconds</t>
+  </si>
+  <si>
+    <t>DissipationSeconds</t>
+  </si>
+  <si>
+    <t>WM01导弹命中后的即时球形法术场；伤害、范围和时序均在本行配置</t>
+  </si>
+  <si>
+    <t>Instant</t>
+  </si>
+  <si>
+    <t>PointRole</t>
+  </si>
+  <si>
+    <t>PointIndex</t>
+  </si>
+  <si>
+    <t>SocketName</t>
+  </si>
+  <si>
+    <t>OffsetX</t>
+  </si>
+  <si>
+    <t>OffsetY</t>
+  </si>
+  <si>
+    <t>OffsetZ</t>
+  </si>
+  <si>
+    <t>bCalibrated</t>
+  </si>
+  <si>
+    <t>FourFRobot_AimTarget</t>
+  </si>
+  <si>
+    <t>FourFRobot 被攻击时的视觉瞄准点；来自 FX_AimTarget</t>
+  </si>
+  <si>
+    <t>AimTarget</t>
+  </si>
+  <si>
+    <t>FX_AimTarget</t>
+  </si>
+  <si>
+    <t>FourFRobot_BasicAttack_Muzzle_0</t>
+  </si>
+  <si>
+    <t>FourFRobot 机枪枪口；来自 FX_Muzzle_Basic_01</t>
+  </si>
+  <si>
+    <t>Muzzle</t>
+  </si>
+  <si>
+    <t>FX_Muzzle_Basic_01</t>
+  </si>
+  <si>
+    <t>WM01_AimTarget</t>
+  </si>
+  <si>
+    <t>WM01 被攻击时的视觉瞄准点；来自 FX_AimTarget</t>
+  </si>
+  <si>
+    <t>WM01_BasicAttack_Muzzle_0</t>
+  </si>
+  <si>
+    <t>WM01 前机枪枪口；来自 FX_Muzzle_Basic_01</t>
+  </si>
+  <si>
+    <t>WM01_MissileLauncher_Muzzle_0</t>
+  </si>
+  <si>
+    <t>WM01 导弹发射口 1；来自 FX_Missile_01</t>
+  </si>
+  <si>
+    <t>FX_Missile_01</t>
+  </si>
+  <si>
+    <t>WM01_MissileLauncher_Muzzle_1</t>
+  </si>
+  <si>
+    <t>WM01 导弹发射口 2；来自 FX_Missile_02</t>
+  </si>
+  <si>
+    <t>FX_Missile_02</t>
   </si>
 </sst>
 </file>
@@ -188,7 +349,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -198,6 +359,21 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEAF2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDEDED"/>
       </patternFill>
     </fill>
   </fills>
@@ -227,10 +403,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="false">
+      <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="true" applyBorder="true" applyAlignment="true">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
+      <alignment vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -604,10 +798,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D5">
         <v>3600</v>
@@ -616,7 +810,7 @@
         <v>300.5</v>
       </c>
       <c r="F5" t="s">
-        <v>18</v>
+        <v>53</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -652,6 +846,9 @@
       <c r="G1" t="s">
         <v>25</v>
       </c>
+      <c r="H1" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -675,6 +872,9 @@
       <c r="G2" t="s">
         <v>10</v>
       </c>
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -698,6 +898,9 @@
       <c r="G3" t="s">
         <v>13</v>
       </c>
+      <c r="H3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -707,7 +910,7 @@
         <v>26</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
         <v>26</v>
@@ -720,6 +923,9 @@
       </c>
       <c r="G4" t="s">
         <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="5">
@@ -743,6 +949,35 @@
       </c>
       <c r="G5" t="s">
         <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G6" t="s">
+        <v>63</v>
+      </c>
+      <c r="H6" t="s">
+        <v>69</v>
       </c>
     </row>
   </sheetData>
@@ -886,10 +1121,10 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -950,10 +1185,10 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
       <c r="D7">
         <v>2</v>
@@ -975,6 +1210,536 @@
       </c>
       <c r="J7">
         <v>18000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" t="s">
+        <v>70</v>
+      </c>
+      <c r="D8">
+        <v>2</v>
+      </c>
+      <c r="E8" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" t="s">
+        <v>59</v>
+      </c>
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="J8">
+        <v>15000</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="2" min="2" width="28"/>
+    <col customWidth="true" max="3" min="3" width="56"/>
+    <col customWidth="true" max="10" min="4" width="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="4">
+        <v>30</v>
+      </c>
+      <c r="E4" s="4">
+        <v>800</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="4">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4">
+        <v>0</v>
+      </c>
+      <c r="I4" s="4">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="1" min="1" width="8"/>
+    <col customWidth="true" max="2" min="2" width="40"/>
+    <col customWidth="true" max="3" min="3" width="48"/>
+    <col customWidth="true" max="4" min="4" width="12"/>
+    <col customWidth="true" max="5" min="5" width="20"/>
+    <col customWidth="true" max="6" min="6" width="14"/>
+    <col customWidth="true" max="7" min="7" width="12"/>
+    <col customWidth="true" max="8" min="8" width="28"/>
+    <col customWidth="true" max="12" min="9" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="true">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7">
+        <v>1</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="7">
+        <v>1</v>
+      </c>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G4" s="7">
+        <v>0</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="I4" s="7">
+        <v>0</v>
+      </c>
+      <c r="J4" s="7">
+        <v>0</v>
+      </c>
+      <c r="K4" s="7">
+        <v>650</v>
+      </c>
+      <c r="L4" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7">
+        <v>2</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="7">
+        <v>1</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G5" s="7">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="7">
+        <v>-480</v>
+      </c>
+      <c r="J5" s="7">
+        <v>5</v>
+      </c>
+      <c r="K5" s="7">
+        <v>935</v>
+      </c>
+      <c r="L5" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7">
+        <v>3</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="D6" s="7">
+        <v>2</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="F6" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="G6" s="7">
+        <v>0</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="I6" s="7">
+        <v>0</v>
+      </c>
+      <c r="J6" s="7">
+        <v>495</v>
+      </c>
+      <c r="K6" s="7">
+        <v>1600</v>
+      </c>
+      <c r="L6" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7">
+        <v>4</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="7">
+        <v>2</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="7">
+        <v>0</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="I7" s="7">
+        <v>1490</v>
+      </c>
+      <c r="J7" s="7">
+        <v>466</v>
+      </c>
+      <c r="K7" s="7">
+        <v>1810</v>
+      </c>
+      <c r="L7" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7">
+        <v>5</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D8" s="7">
+        <v>2</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G8" s="7">
+        <v>0</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="I8" s="7">
+        <v>-260</v>
+      </c>
+      <c r="J8" s="7">
+        <v>1257</v>
+      </c>
+      <c r="K8" s="7">
+        <v>2440</v>
+      </c>
+      <c r="L8" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" s="7">
+        <v>2</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="G9" s="7">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="I9" s="7">
+        <v>-260</v>
+      </c>
+      <c r="J9" s="7">
+        <v>-326</v>
+      </c>
+      <c r="K9" s="7">
+        <v>2440</v>
+      </c>
+      <c r="L9" s="7" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement commander strongholds and airborne engineering transit
Add table-driven buildings, component-based construction and ownership,
first-capture facilities, atomic upkeep, shields, production, and population
reservations. Share airborne travel between mining and construction vehicles
with deterministic topology, phase replication, safe exits, and blue VFX.

Include Excel sources, generated data, assets, documentation, and PIE evidence.
Source UE5.7 Editor and Game builds pass with matching BuildId. Resource and
damage-ledger regressions and placement policy pass; two legacy building tests
still fail against old contracts, and the 600-unit run remains slow.
No automation test code was added or changed.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
   <si>
     <t>id</t>
   </si>
@@ -395,6 +395,18 @@
   </si>
   <si>
     <t>/Game/GuLiStrike/Vehicles/ElectromagneticMiner/BP_MiningVehicle_TransporterLvl2.BP_MiningVehicle_TransporterLvl2_C</t>
+  </si>
+  <si>
+    <t>ConstructionVehicle</t>
+  </si>
+  <si>
+    <t>开局每队一辆；独立建造车，施工与采矿分工</t>
+  </si>
+  <si>
+    <t>/Script/GuLiStrike.GuLiConstructionVehiclePawn</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Vehicles/ConstructionVehicle/BP_ConstructionVehicle.BP_ConstructionVehicle_C</t>
   </si>
 </sst>
 </file>
@@ -958,6 +970,38 @@
         <v>3.0422898572084356</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>127</v>
+      </c>
+      <c r="C7" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7">
+        <v>4500</v>
+      </c>
+      <c r="E7">
+        <v>1000</v>
+      </c>
+      <c r="F7" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I7" t="s">
+        <v>130</v>
+      </c>
+      <c r="J7">
+        <v>3.0422898572084356</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: back up commander optimizations, navigation, and art updates
Back up commander pose compression and client CPU/GPU presentation updates.
Include engineering crowd avoidance, navigation pre-baking, and engine patch sources.
Sync stylized model and explosion assets, tables, authoring scripts, progress
records, and recorded verification and profiling evidence.

Keep new marketplace source packs and cooked outputs local, and store TGA
art textures with Git LFS.

Pre-push checks: documentation indexes current; documentation check has zero
errors; staged LFS pointers and local objects verified; no oversized ordinary
Git blobs. Preserve original generated evidence and patch formatting.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="137">
   <si>
     <t>id</t>
   </si>
@@ -407,6 +407,24 @@
   </si>
   <si>
     <t>/Game/GuLiStrike/Vehicles/ConstructionVehicle/BP_ConstructionVehicle.BP_ConstructionVehicle_C</t>
+  </si>
+  <si>
+    <t>扫荡者</t>
+  </si>
+  <si>
+    <t>战争机器</t>
+  </si>
+  <si>
+    <t>电磁矿车</t>
+  </si>
+  <si>
+    <t>建造车</t>
+  </si>
+  <si>
+    <t>/Game/Commander/Units/Tactical/Cel/Sweeper/Meshes/SM_Sweeper_Cel.SM_Sweeper_Cel</t>
+  </si>
+  <si>
+    <t>/Game/Commander/Units/Tactical/Cel/WarMachine/Meshes/SM_WarMachine_Cel.SM_WarMachine_Cel</t>
   </si>
 </sst>
 </file>
@@ -809,6 +827,9 @@
       <c r="J1" t="s">
         <v>121</v>
       </c>
+      <c r="K1" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -841,6 +862,9 @@
       <c r="J2" t="s">
         <v>11</v>
       </c>
+      <c r="K2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -873,6 +897,9 @@
       <c r="J3" t="s">
         <v>13</v>
       </c>
+      <c r="K3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -891,7 +918,7 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>135</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -904,6 +931,9 @@
       </c>
       <c r="J4">
         <v>1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="5">
@@ -923,7 +953,7 @@
         <v>300.5</v>
       </c>
       <c r="F5" t="s">
-        <v>53</v>
+        <v>136</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -936,6 +966,9 @@
       </c>
       <c r="J5">
         <v>1</v>
+      </c>
+      <c r="K5" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="6">
@@ -969,6 +1002,9 @@
       <c r="J6">
         <v>3.0422898572084356</v>
       </c>
+      <c r="K6" t="s">
+        <v>133</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1001,6 +1037,9 @@
       <c r="J7">
         <v>3.0422898572084356</v>
       </c>
+      <c r="K7" t="s">
+        <v>134</v>
+      </c>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>

<commit_message>
feat: integrate ground mechs and combat updates
Add the ground mech runtime and production asset set, update commander unit sizing and navigation behavior, revise WM01 missile ranges and explosion presentation, and archive the associated validation evidence. Clean local session artifacts and retain versioned documentation entry points.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -13,8 +13,28 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>GuLiStrike</author>
+  </authors>
+  <commentList>
+    <comment ref="L1" authorId="0">
+      <text>
+        <t>模型宽度，单位：米。最终游戏尺度下用于平面圆形占地的直径。代码接入时半径=宽度×50厘米，不再乘PresentationScale，也不修改模型缩放。战争机器12.5米由用户指定；扫荡者按实测水平尺寸向上取3.1米；两种工程车按当前3.6米车长取值。</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0">
+      <text>
+        <t>最小避障距离，单位：米。两个单位圆形占地外缘之间的最小净距，不是中心距离。双方取较大值，不相加。最小中心距=(A模型宽度+B模型宽度)/2+max(A最小避障距离,B最小避障距离)。战争机器之间为15米。本次仅完成源表配置，运行时代码尚待接入。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
   <si>
     <t>id</t>
   </si>
@@ -428,12 +448,21 @@
   </si>
   <si>
     <t>指挥官可控制矿车；Scale020后车长3.6米，900cm/s；采矿业务由矿车Manager调度</t>
+  </si>
+  <si>
+    <t>ModelWidthMeters</t>
+  </si>
+  <si>
+    <t>MinAvoidanceDistanceMeters</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0&quot; m&quot;"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -501,7 +530,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -523,6 +552,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="true" applyAlignment="true">
       <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
+      <alignment/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -790,13 +822,15 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <dimension ref="A1"/>
   <cols>
     <col customWidth="true" max="1" min="1" width="10"/>
     <col customWidth="true" max="2" min="2" width="22"/>
     <col customWidth="true" max="3" min="3" width="46"/>
     <col customWidth="true" max="7" min="4" width="28"/>
+    <col customWidth="true" max="12" min="12" width="26"/>
+    <col customWidth="true" max="13" min="13" width="35"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -833,6 +867,12 @@
       <c r="K1" t="s">
         <v>23</v>
       </c>
+      <c r="L1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M1" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -868,6 +908,12 @@
       <c r="K2" t="s">
         <v>10</v>
       </c>
+      <c r="L2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -903,6 +949,12 @@
       <c r="K3" t="s">
         <v>14</v>
       </c>
+      <c r="L3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -938,6 +990,12 @@
       <c r="K4" t="s">
         <v>131</v>
       </c>
+      <c r="L4" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="M4" s="8">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -973,6 +1031,12 @@
       <c r="K5" t="s">
         <v>132</v>
       </c>
+      <c r="L5" s="8">
+        <v>12.5</v>
+      </c>
+      <c r="M5" s="8">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1008,6 +1072,12 @@
       <c r="K6" t="s">
         <v>133</v>
       </c>
+      <c r="L6" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="M6" s="8">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1043,7 +1113,14 @@
       <c r="K7" t="s">
         <v>134</v>
       </c>
+      <c r="L7" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="M7" s="8">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: update Mass movement, commander gameplay and project assets
Implement immediate Mass movement with shared NavMesh routes, command-wide random slots, incremental state delivery and persistent route lines.
Integrate commander StateTree behaviors, construction and resource workflows, map authoring updates, card demo assets and data pipeline changes.
Include development and player acceptance records while keeping generated map backups, terrain buffers and raw profiling captures local.

Validation: source UE 5.7 GuLiStrikeEditor Win64 Development build and module BuildIds verified; Mass PIE response and slot data sampled; player accepted the resulting behavior. Staged source whitespace and LFS checks passed.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
   <si>
     <t>id</t>
   </si>
@@ -454,6 +454,18 @@
   </si>
   <si>
     <t>MinAvoidanceDistanceMeters</t>
+  </si>
+  <si>
+    <t>StateTreeAsset</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Commander/Behavior/ST_CommanderMass.ST_CommanderMass</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Commander/Behavior/ST_CommanderMiner.ST_CommanderMiner</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Commander/Behavior/ST_CommanderBuilder.ST_CommanderBuilder</t>
   </si>
 </sst>
 </file>
@@ -831,6 +843,7 @@
     <col customWidth="true" max="7" min="4" width="28"/>
     <col customWidth="true" max="12" min="12" width="26"/>
     <col customWidth="true" max="13" min="13" width="35"/>
+    <col customWidth="true" max="14" min="14" width="58"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -873,6 +886,9 @@
       <c r="M1" t="s">
         <v>139</v>
       </c>
+      <c r="N1" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -914,6 +930,9 @@
       <c r="M2" t="s">
         <v>11</v>
       </c>
+      <c r="N2" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -955,6 +974,9 @@
       <c r="M3" t="s">
         <v>13</v>
       </c>
+      <c r="N3" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4">
@@ -996,6 +1018,9 @@
       <c r="M4" s="8">
         <v>0.5</v>
       </c>
+      <c r="N4" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5">
@@ -1037,6 +1062,9 @@
       <c r="M5" s="8">
         <v>2.5</v>
       </c>
+      <c r="N5" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1078,6 +1106,9 @@
       <c r="M6" s="8">
         <v>1</v>
       </c>
+      <c r="N6" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1118,6 +1149,9 @@
       </c>
       <c r="M7" s="8">
         <v>1</v>
+      </c>
+      <c r="N7" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: integrate commander LOD, WM01 visuals and rogue card updates
Add the shared three-level commander LOD service and migrate missile
presentation, with GPU smoke history, budget reporting and candidate assets.
Include accumulated WM01 mechanical animation, hover, missile unlock/card,
UI, data, authoring tools and project documentation changes.

Retain source assets and validation evidence, move this LOD session's ten
temporary files to recoverable storage outside the project, and exclude
editor recovery maps while preserving the existing large-map ignore rules.

Validation: documentation build/check reports zero errors (13 existing
warnings); all changed UE binary assets are LFS pointers. Earlier limited
PIE observations used 36/37 units; the later fixture source fix still needs
a build and revalidation. No new build, PIE or performance run for this sync.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
   <si>
     <t>id</t>
   </si>
@@ -466,6 +466,15 @@
   </si>
   <si>
     <t>/Game/GuLiStrike/Commander/Behavior/ST_CommanderBuilder.ST_CommanderBuilder</t>
+  </si>
+  <si>
+    <t>/Game/Commander/Units/Tactical/Cel/Sweeper/Meshes/SM_Sweeper_Rigid.SM_Sweeper_Rigid</t>
+  </si>
+  <si>
+    <t>/Game/Commander/Units/Tactical/Cel/WarMachine/Meshes/SM_WarMachine_Rigid.SM_WarMachine_Rigid</t>
+  </si>
+  <si>
+    <t>重防号</t>
   </si>
 </sst>
 </file>
@@ -995,7 +1004,7 @@
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1039,7 +1048,7 @@
         <v>300.5</v>
       </c>
       <c r="F5" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1054,7 +1063,7 @@
         <v>0.2</v>
       </c>
       <c r="K5" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="L5" s="8">
         <v>12.5</v>

</xml_diff>

<commit_message>
feat: deliver Pioneer generation one and flight event networking
Record user approval and preserve B-v1 art sources, VAT delivery, dual guns and Q summons. Integrate batched projectile lifecycle events, client visual pools and real-time connection budget accounting with the compiled shared Commander/table/asset baseline and acceptance evidence. Reviewed temporary files remain local because automatic approval blocked deletion; exclude all 55 from this delivery.
</commit_message>
<xml_diff>
--- a/data/Excel/GuLiStrikeCommander.xlsx
+++ b/data/Excel/GuLiStrikeCommander.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="true" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14805" windowHeight="8010" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Soldiers" sheetId="2" r:id="rId4"/>
+    <sheet name="Camera" sheetId="3" r:id="rId6"/>
   </sheets>
   <calcPr calcId="122211"/>
 </workbook>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="188">
   <si>
     <t>id</t>
   </si>
@@ -475,6 +476,129 @@
   </si>
   <si>
     <t>重防号</t>
+  </si>
+  <si>
+    <t>Default</t>
+  </si>
+  <si>
+    <t>三档镜头；距离米、俯角向下为正、时间秒。x由战场和HUD可用画面计算；数值修改后导出并导入Camera表。</t>
+  </si>
+  <si>
+    <t>MinimumHeightMeters</t>
+  </si>
+  <si>
+    <t>TacticalStartHeightMeters</t>
+  </si>
+  <si>
+    <t>TacticalMaximumHeightMeters</t>
+  </si>
+  <si>
+    <t>InitialHeightMeters</t>
+  </si>
+  <si>
+    <t>NearPitchDegrees</t>
+  </si>
+  <si>
+    <t>TacticalPitchDegrees</t>
+  </si>
+  <si>
+    <t>OverviewPitchDegrees</t>
+  </si>
+  <si>
+    <t>FieldOfViewDegrees</t>
+  </si>
+  <si>
+    <t>ZoomStepMultiplier</t>
+  </si>
+  <si>
+    <t>ZoomInterpolationSpeed</t>
+  </si>
+  <si>
+    <t>YawDegreesPerSecond</t>
+  </si>
+  <si>
+    <t>MoveHeightMultiplier</t>
+  </si>
+  <si>
+    <t>MinimumMoveMetersPerSecond</t>
+  </si>
+  <si>
+    <t>MaximumMoveMetersPerSecond</t>
+  </si>
+  <si>
+    <t>RiseHalfLifeSeconds</t>
+  </si>
+  <si>
+    <t>DescentHalfLifeSeconds</t>
+  </si>
+  <si>
+    <t>MaximumRiseMetersPerSecond</t>
+  </si>
+  <si>
+    <t>MaximumDescentMetersPerSecond</t>
+  </si>
+  <si>
+    <t>LookAheadSeconds</t>
+  </si>
+  <si>
+    <t>BoundaryPaddingMeters</t>
+  </si>
+  <si>
+    <t>PivotClearanceMeters</t>
+  </si>
+  <si>
+    <t>BoomClearanceMeters</t>
+  </si>
+  <si>
+    <t>CameraClearanceMeters</t>
+  </si>
+  <si>
+    <t>BoomSampleSpacingMeters</t>
+  </si>
+  <si>
+    <t>OverviewTransitionSeconds</t>
+  </si>
+  <si>
+    <t>OverviewPaddingFraction</t>
+  </si>
+  <si>
+    <t>OverviewUnitIconPixels</t>
+  </si>
+  <si>
+    <t>OverviewBuildingIconPixels</t>
+  </si>
+  <si>
+    <t>ZoomInterpolationPerSecond</t>
+  </si>
+  <si>
+    <t>MoveHeightMultiplierPerSecond</t>
+  </si>
+  <si>
+    <t>OverviewYawDegrees</t>
+  </si>
+  <si>
+    <t>VATDefinition</t>
+  </si>
+  <si>
+    <t>bSummonOnly</t>
+  </si>
+  <si>
+    <t>B-v1先驱号；6.25米；刚性骨骼纹理VAT；默认双枪与Q召唤</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Robots/RSGMech/Meshes/SM_Pioneer_VAT.SM_Pioneer_VAT</t>
+  </si>
+  <si>
+    <t>先驱号</t>
+  </si>
+  <si>
+    <t>/Game/GuLiStrike/Robots/RSGMech/VAT/DA_Pioneer_VAT.DA_Pioneer_VAT</t>
+  </si>
+  <si>
+    <t>SweeperSummon</t>
+  </si>
+  <si>
+    <t>先驱号Q专用召唤兵；永久可控、可累积、不计生产人口</t>
   </si>
 </sst>
 </file>
@@ -551,7 +675,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="true" applyFill="true" applyBorder="true" applyAlignment="true">
       <alignment horizontal="center"/>
@@ -576,6 +700,12 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="true" applyAlignment="false">
       <alignment/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="true" applyFill="true" applyAlignment="true">
+      <alignment wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment wrapText="true"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -898,6 +1028,12 @@
       <c r="N1" t="s">
         <v>140</v>
       </c>
+      <c r="O1" t="s">
+        <v>180</v>
+      </c>
+      <c r="P1" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
@@ -942,6 +1078,12 @@
       <c r="N2" t="s">
         <v>12</v>
       </c>
+      <c r="O2" t="s">
+        <v>12</v>
+      </c>
+      <c r="P2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
@@ -985,6 +1127,12 @@
       </c>
       <c r="N3" t="s">
         <v>13</v>
+      </c>
+      <c r="O3" t="s">
+        <v>14</v>
+      </c>
+      <c r="P3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -995,16 +1143,16 @@
         <v>15</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>182</v>
       </c>
       <c r="D4">
-        <v>720</v>
+        <v>1440</v>
       </c>
       <c r="E4">
         <v>100</v>
       </c>
       <c r="F4" t="s">
-        <v>144</v>
+        <v>183</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1016,19 +1164,25 @@
         <v>68</v>
       </c>
       <c r="J4">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="K4" t="s">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="L4" s="8">
-        <v>3.1</v>
+        <v>6.25</v>
       </c>
       <c r="M4" s="8">
         <v>0.5</v>
       </c>
       <c r="N4" t="s">
         <v>141</v>
+      </c>
+      <c r="O4" t="s">
+        <v>185</v>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -1074,6 +1228,9 @@
       <c r="N5" t="s">
         <v>141</v>
       </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6">
@@ -1118,6 +1275,9 @@
       <c r="N6" t="s">
         <v>142</v>
       </c>
+      <c r="P6" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7">
@@ -1162,8 +1322,456 @@
       <c r="N7" t="s">
         <v>143</v>
       </c>
+      <c r="P7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>186</v>
+      </c>
+      <c r="C8" t="s">
+        <v>187</v>
+      </c>
+      <c r="D8">
+        <v>720</v>
+      </c>
+      <c r="E8">
+        <v>100</v>
+      </c>
+      <c r="F8" t="s">
+        <v>144</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0.2</v>
+      </c>
+      <c r="K8" t="s">
+        <v>131</v>
+      </c>
+      <c r="L8">
+        <v>3.1</v>
+      </c>
+      <c r="M8">
+        <v>0.5</v>
+      </c>
+      <c r="N8" t="s">
+        <v>141</v>
+      </c>
+      <c r="P8" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1"/>
+  <cols>
+    <col customWidth="true" max="3" min="3" width="55"/>
+    <col customWidth="true" max="32" min="4" width="24"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="true">
+      <c r="A1" s="9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>150</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>152</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>153</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>178</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="Q1" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="R1" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="S1" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="T1" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="U1" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="V1" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="W1" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="X1" s="9" t="s">
+        <v>169</v>
+      </c>
+      <c r="Y1" s="9" t="s">
+        <v>170</v>
+      </c>
+      <c r="Z1" s="9" t="s">
+        <v>171</v>
+      </c>
+      <c r="AA1" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="AB1" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="AC1" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="AD1" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="AE1" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF1" s="9" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N2" t="s">
+        <v>11</v>
+      </c>
+      <c r="O2" t="s">
+        <v>11</v>
+      </c>
+      <c r="P2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>11</v>
+      </c>
+      <c r="R2" t="s">
+        <v>11</v>
+      </c>
+      <c r="S2" t="s">
+        <v>11</v>
+      </c>
+      <c r="T2" t="s">
+        <v>11</v>
+      </c>
+      <c r="U2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V2" t="s">
+        <v>11</v>
+      </c>
+      <c r="W2" t="s">
+        <v>11</v>
+      </c>
+      <c r="X2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>11</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E3" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" t="s">
+        <v>13</v>
+      </c>
+      <c r="N3" t="s">
+        <v>13</v>
+      </c>
+      <c r="O3" t="s">
+        <v>13</v>
+      </c>
+      <c r="P3" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R3" t="s">
+        <v>13</v>
+      </c>
+      <c r="S3" t="s">
+        <v>13</v>
+      </c>
+      <c r="T3" t="s">
+        <v>13</v>
+      </c>
+      <c r="U3" t="s">
+        <v>13</v>
+      </c>
+      <c r="V3" t="s">
+        <v>13</v>
+      </c>
+      <c r="W3" t="s">
+        <v>13</v>
+      </c>
+      <c r="X3" t="s">
+        <v>13</v>
+      </c>
+      <c r="Y3" t="s">
+        <v>13</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AE3" t="s">
+        <v>13</v>
+      </c>
+      <c r="AF3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" ht="60" customHeight="true">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="D4">
+        <v>35</v>
+      </c>
+      <c r="E4">
+        <v>300</v>
+      </c>
+      <c r="F4">
+        <v>700</v>
+      </c>
+      <c r="G4">
+        <v>133.4</v>
+      </c>
+      <c r="H4">
+        <v>25</v>
+      </c>
+      <c r="I4">
+        <v>55</v>
+      </c>
+      <c r="J4">
+        <v>90</v>
+      </c>
+      <c r="K4">
+        <v>45</v>
+      </c>
+      <c r="L4">
+        <v>1.18</v>
+      </c>
+      <c r="M4">
+        <v>8</v>
+      </c>
+      <c r="N4">
+        <v>70</v>
+      </c>
+      <c r="O4">
+        <v>1.4</v>
+      </c>
+      <c r="P4">
+        <v>12</v>
+      </c>
+      <c r="Q4">
+        <v>92</v>
+      </c>
+      <c r="R4">
+        <v>0.2</v>
+      </c>
+      <c r="S4">
+        <v>0.35</v>
+      </c>
+      <c r="T4">
+        <v>60</v>
+      </c>
+      <c r="U4">
+        <v>30</v>
+      </c>
+      <c r="V4">
+        <v>0.75</v>
+      </c>
+      <c r="W4">
+        <v>10</v>
+      </c>
+      <c r="X4">
+        <v>0.3</v>
+      </c>
+      <c r="Y4">
+        <v>0.4</v>
+      </c>
+      <c r="Z4">
+        <v>1</v>
+      </c>
+      <c r="AA4">
+        <v>20</v>
+      </c>
+      <c r="AB4">
+        <v>0.6</v>
+      </c>
+      <c r="AC4">
+        <v>0.05</v>
+      </c>
+      <c r="AD4">
+        <v>14</v>
+      </c>
+      <c r="AE4">
+        <v>20</v>
+      </c>
+      <c r="AF4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>